<commit_message>
fix : bugs on project charter and gantt excel.
</commit_message>
<xml_diff>
--- a/02_Documentazione_Progetto/02_Planning/04_Tempi_Costi_e_Gantt_TrailSafe.xlsx
+++ b/02_Documentazione_Progetto/02_Planning/04_Tempi_Costi_e_Gantt_TrailSafe.xlsx
@@ -3526,8 +3526,8 @@
         <v>98</v>
       </c>
       <c r="J23" s="20">
-        <f>SUM(J6:J21)</f>
-        <v>72400</v>
+        <f>Costi!B16</f>
+        <v>67980</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>

</xml_diff>